<commit_message>
abandoned carts: monthly 2026-10-03
</commit_message>
<xml_diff>
--- a/reports/abandoned-carts/abandoned_carts_monthly_2026-09-01_2026-09-30.xlsx
+++ b/reports/abandoned-carts/abandoned_carts_monthly_2026-09-01_2026-09-30.xlsx
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J30" s="9">
         <f>G30+H30+I30</f>
@@ -2046,7 +2046,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>176034</v>
+        <v>150024</v>
       </c>
       <c r="N30" s="8">
         <f>K30+L30+M30</f>
@@ -2285,7 +2285,7 @@
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>How this was built (Shopify Admin API, pulled 03 Oct 2026 14:25 IST; blue = pulled values, black = formulas):</t>
+          <t>How this was built (Shopify Admin API, pulled 03 Oct 2026 15:38 IST; blue = pulled values, black = formulas):</t>
         </is>
       </c>
     </row>
@@ -4316,7 +4316,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" s="5" t="n">
         <v>0</v>
@@ -4338,7 +4338,7 @@
         <v>0</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>176034</v>
+        <v>150024</v>
       </c>
       <c r="M30" s="6" t="n">
         <v>0</v>
@@ -4358,7 +4358,7 @@
         <v/>
       </c>
       <c r="R30" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S30" s="5" t="n">
         <v>0</v>

</xml_diff>